<commit_message>
update ukom and it's flows
</commit_message>
<xml_diff>
--- a/storage/app/buckets/template/template_grade.xlsx
+++ b/storage/app/buckets/template/template_grade.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28521"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29010"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\EyeGil\_LARAVEL\be-template-laravel\storage\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{7284FCF7-6AB5-45AA-95FF-FE517488C5FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A7B521B-DF99-424E-820F-D861B47FB522}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{7284FCF7-6AB5-45AA-95FF-FE517488C5FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA82D93C-A519-4951-B938-B0945B477A06}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{7C472A89-B406-4666-A45E-95F23D99CBAE}"/>
   </bookViews>
@@ -36,9 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>NIP/Email</t>
+  </si>
+  <si>
+    <t>Nilai CAT</t>
   </si>
   <si>
     <t>Nilai Wawancara</t>
@@ -93,13 +96,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF272A3A"/>
+      <name val="Public Sans"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -122,13 +132,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -142,26 +158,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06EDFEEE-1947-4334-9ACA-EB9182AAA23C}" name="Table2" displayName="Table2" ref="A1:Q2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:Q2" xr:uid="{06EDFEEE-1947-4334-9ACA-EB9182AAA23C}"/>
-  <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{CCFAB820-A083-4907-A62C-A8A3C822968F}" name="NIP/Email"/>
-    <tableColumn id="2" xr3:uid="{A25DBFED-888B-4793-9B9F-5A21F0A25E8E}" name="Nilai Wawancara"/>
-    <tableColumn id="3" xr3:uid="{06F0E890-7437-45DE-AD51-D86814E61131}" name="Nilai Seminar"/>
-    <tableColumn id="4" xr3:uid="{CDEE73F8-161C-40CA-93BA-DE0329EB0371}" name="Nilai Praktik"/>
-    <tableColumn id="5" xr3:uid="{BE5ADE43-B2C7-4586-A6C4-019931DB03F3}" name="Nilai Portofolia"/>
-    <tableColumn id="6" xr3:uid="{2C254BDA-EDBD-4796-B3A5-CBFD766439DB}" name="Nilai Integritas"/>
-    <tableColumn id="7" xr3:uid="{C3E726A2-8187-4F66-8936-8808634BF2B3}" name="Nilai Kerja Sama"/>
-    <tableColumn id="8" xr3:uid="{F1317D23-2CD6-48D8-B847-5D3D21FA90BE}" name="Nilai Komunikasi"/>
-    <tableColumn id="9" xr3:uid="{D1C94BCA-9D89-4A9F-A1C7-456EBC88DD33}" name="Nilai Orientasi"/>
-    <tableColumn id="10" xr3:uid="{24504279-EFB3-49C8-9A45-DBF716606C81}" name="Nilai Pelayanan Publik"/>
-    <tableColumn id="11" xr3:uid="{156BD834-D178-4FCC-97F9-A6D53C381443}" name="Nilai Pengembangan Diri"/>
-    <tableColumn id="12" xr3:uid="{385066C5-259A-404D-AE33-D83C8A46843D}" name="Nilai Mengelola Perubahan"/>
-    <tableColumn id="13" xr3:uid="{9289009B-8B4C-442F-A981-61B7ECF3A50E}" name="Nilai Pengambilan Keputusan"/>
-    <tableColumn id="14" xr3:uid="{F503B227-AF19-481D-9A2F-2B1AE422764C}" name="Nilai Perekat Bangsa"/>
-    <tableColumn id="15" xr3:uid="{71A1A061-0D65-4C4D-A807-7B0282A2CE16}" name="Score"/>
-    <tableColumn id="16" xr3:uid="{4CF8380C-7852-4D4A-8A16-1596E6EB1F3A}" name="JPM"/>
-    <tableColumn id="17" xr3:uid="{F552C85E-6668-4225-A327-FEF0FBD02890}" name="Kategori"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06EDFEEE-1947-4334-9ACA-EB9182AAA23C}" name="Table2" displayName="Table2" ref="A1:R4" totalsRowShown="0">
+  <autoFilter ref="A1:R4" xr:uid="{06EDFEEE-1947-4334-9ACA-EB9182AAA23C}"/>
+  <tableColumns count="18">
+    <tableColumn id="1" xr3:uid="{CCFAB820-A083-4907-A62C-A8A3C822968F}" name="NIP/Email" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{A25DBFED-888B-4793-9B9F-5A21F0A25E8E}" name="Nilai CAT"/>
+    <tableColumn id="3" xr3:uid="{06F0E890-7437-45DE-AD51-D86814E61131}" name="Nilai Wawancara"/>
+    <tableColumn id="4" xr3:uid="{CDEE73F8-161C-40CA-93BA-DE0329EB0371}" name="Nilai Seminar"/>
+    <tableColumn id="5" xr3:uid="{BE5ADE43-B2C7-4586-A6C4-019931DB03F3}" name="Nilai Praktik"/>
+    <tableColumn id="6" xr3:uid="{2C254BDA-EDBD-4796-B3A5-CBFD766439DB}" name="Nilai Portofolia"/>
+    <tableColumn id="7" xr3:uid="{C3E726A2-8187-4F66-8936-8808634BF2B3}" name="Nilai Integritas"/>
+    <tableColumn id="8" xr3:uid="{F1317D23-2CD6-48D8-B847-5D3D21FA90BE}" name="Nilai Kerja Sama"/>
+    <tableColumn id="9" xr3:uid="{D1C94BCA-9D89-4A9F-A1C7-456EBC88DD33}" name="Nilai Komunikasi"/>
+    <tableColumn id="10" xr3:uid="{24504279-EFB3-49C8-9A45-DBF716606C81}" name="Nilai Orientasi"/>
+    <tableColumn id="11" xr3:uid="{156BD834-D178-4FCC-97F9-A6D53C381443}" name="Nilai Pelayanan Publik"/>
+    <tableColumn id="12" xr3:uid="{385066C5-259A-404D-AE33-D83C8A46843D}" name="Nilai Pengembangan Diri"/>
+    <tableColumn id="13" xr3:uid="{9289009B-8B4C-442F-A981-61B7ECF3A50E}" name="Nilai Mengelola Perubahan"/>
+    <tableColumn id="14" xr3:uid="{F503B227-AF19-481D-9A2F-2B1AE422764C}" name="Nilai Pengambilan Keputusan"/>
+    <tableColumn id="15" xr3:uid="{71A1A061-0D65-4C4D-A807-7B0282A2CE16}" name="Nilai Perekat Bangsa"/>
+    <tableColumn id="16" xr3:uid="{4CF8380C-7852-4D4A-8A16-1596E6EB1F3A}" name="Score"/>
+    <tableColumn id="17" xr3:uid="{F552C85E-6668-4225-A327-FEF0FBD02890}" name="JPM"/>
+    <tableColumn id="18" xr3:uid="{499B8DC8-4BBD-41E4-9449-62D5B37D9F48}" name="Kategori"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -464,10 +481,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FC5C7B4-97A9-43D3-B093-E46AC961D3C5}">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -486,8 +503,8 @@
     <col min="17" max="17" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
-      <c r="A1" t="s">
+    <row r="1" spans="1:18">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -538,6 +555,12 @@
       <c r="Q1" t="s">
         <v>16</v>
       </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="15">
+      <c r="A3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>